<commit_message>
Improve V2 evaluation and knowledge selection
</commit_message>
<xml_diff>
--- a/evaluation-source/V2评测集模板.xlsx
+++ b/evaluation-source/V2评测集模板.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测案例" sheetId="1" r:id="R558a269d05634440"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R93ed4c28eb1440af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测案例" sheetId="1" r:id="Re578fccca02940ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rb97455acc8764060"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -613,18 +613,21 @@
         <x:v>必须包含</x:v>
       </x:c>
       <x:c r="K1" s="11" t="str">
+        <x:v>任一表达满足</x:v>
+      </x:c>
+      <x:c r="L1" s="11" t="str">
         <x:v>禁止包含</x:v>
       </x:c>
-      <x:c r="L1" s="11" t="str">
+      <x:c r="M1" s="11" t="str">
         <x:v>必须保持原样</x:v>
       </x:c>
-      <x:c r="M1" s="11" t="str">
+      <x:c r="N1" s="11" t="str">
         <x:v>参考回复</x:v>
       </x:c>
-      <x:c r="N1" s="11" t="str">
+      <x:c r="O1" s="12" t="str">
         <x:v>错误类型</x:v>
       </x:c>
-      <x:c r="O1" s="12" t="str">
+      <x:c r="P1" t="str">
         <x:v>备注</x:v>
       </x:c>
     </x:row>
@@ -657,19 +660,20 @@
       <x:c r="J2" s="25" t="str">
         <x:v>POST;/api/v1/environments;env_id</x:v>
       </x:c>
-      <x:c r="K2" s="25" t="str">
+      <x:c r="K2" s="25"/>
+      <x:c r="L2" s="25" t="str">
         <x:v>Local API</x:v>
       </x:c>
-      <x:c r="L2" s="25" t="str">
+      <x:c r="M2" s="25" t="str">
         <x:v>POST;/api/v1/environments;env_id;https://docs.example.test/api/v1/environments</x:v>
       </x:c>
-      <x:c r="M2" s="25" t="str">
+      <x:c r="N2" s="25" t="str">
         <x:v>请使用 POST /api/v1/environments，并保留参数 env_id。</x:v>
       </x:c>
-      <x:c r="N2" s="25" t="str">
+      <x:c r="O2" s="25" t="str">
         <x:v>API类型混淆;Endpoint变化;参数变化</x:v>
       </x:c>
-      <x:c r="O2" s="25" t="str">
+      <x:c r="P2" t="str">
         <x:v>完全脱敏的 HTTP API 示例</x:v>
       </x:c>
     </x:row>
@@ -702,19 +706,20 @@
       <x:c r="J3" s="27" t="str">
         <x:v>Local API;GET;/local/v2/profiles;profile_id</x:v>
       </x:c>
-      <x:c r="K3" s="27" t="str">
+      <x:c r="K3" s="27"/>
+      <x:c r="L3" s="27" t="str">
         <x:v>HTTP API</x:v>
       </x:c>
-      <x:c r="L3" s="27" t="str">
+      <x:c r="M3" s="27" t="str">
         <x:v>GET;/local/v2/profiles;profile_id</x:v>
       </x:c>
-      <x:c r="M3" s="27" t="str">
+      <x:c r="N3" s="27" t="str">
         <x:v>Use GET /local/v2/profiles with profile_id.</x:v>
       </x:c>
-      <x:c r="N3" s="27" t="str">
+      <x:c r="O3" s="27" t="str">
         <x:v>API类型混淆;Method变化</x:v>
       </x:c>
-      <x:c r="O3" s="27" t="str">
+      <x:c r="P3" t="str">
         <x:v>完全脱敏的 Local API 示例</x:v>
       </x:c>
     </x:row>
@@ -747,17 +752,18 @@
       <x:c r="J4" s="27" t="str">
         <x:v>https://help.example.test/start?lang=en#install;/api/v1/status</x:v>
       </x:c>
-      <x:c r="K4" s="27" t="str"/>
-      <x:c r="L4" s="27" t="str">
+      <x:c r="K4" s="27"/>
+      <x:c r="L4" s="27"/>
+      <x:c r="M4" s="27" t="str">
         <x:v>https://help.example.test/start?lang=en#install;/api/v1/status</x:v>
       </x:c>
-      <x:c r="M4" s="27" t="str">
+      <x:c r="N4" s="27" t="str">
         <x:v>Open the setup link, then check /api/v1/status.</x:v>
       </x:c>
-      <x:c r="N4" s="27" t="str">
+      <x:c r="O4" s="27" t="str">
         <x:v>URL变化;Endpoint变化</x:v>
       </x:c>
-      <x:c r="O4" s="27" t="str">
+      <x:c r="P4" t="str">
         <x:v>使用 example.test 保证不指向真实系统</x:v>
       </x:c>
     </x:row>
@@ -790,17 +796,18 @@
       <x:c r="J5" s="27" t="str">
         <x:v>Profile settings;Browser fingerprint</x:v>
       </x:c>
-      <x:c r="K5" s="27" t="str"/>
-      <x:c r="L5" s="27" t="str">
+      <x:c r="K5" s="27"/>
+      <x:c r="L5" s="27"/>
+      <x:c r="M5" s="27" t="str">
         <x:v>Profile settings;Browser fingerprint</x:v>
       </x:c>
-      <x:c r="M5" s="27" t="str">
+      <x:c r="N5" s="27" t="str">
         <x:v>Check Browser fingerprint in Profile settings.</x:v>
       </x:c>
-      <x:c r="N5" s="27" t="str">
+      <x:c r="O5" s="27" t="str">
         <x:v>术语变化</x:v>
       </x:c>
-      <x:c r="O5" s="27" t="str">
+      <x:c r="P5" t="str">
         <x:v>脱敏术语示例</x:v>
       </x:c>
     </x:row>
@@ -833,19 +840,20 @@
       <x:c r="J6" s="27" t="str">
         <x:v>POST;/api/v1/environments;env_id</x:v>
       </x:c>
-      <x:c r="K6" s="27" t="str">
+      <x:c r="K6" s="27"/>
+      <x:c r="L6" s="27" t="str">
         <x:v>Local API</x:v>
       </x:c>
-      <x:c r="L6" s="27" t="str">
+      <x:c r="M6" s="27" t="str">
         <x:v>POST;/api/v1/environments;env_id</x:v>
       </x:c>
-      <x:c r="M6" s="27" t="str">
+      <x:c r="N6" s="27" t="str">
         <x:v>Utilice POST /api/v1/environments con env_id.</x:v>
       </x:c>
-      <x:c r="N6" s="27" t="str">
+      <x:c r="O6" s="27" t="str">
         <x:v>多语言;Endpoint变化</x:v>
       </x:c>
-      <x:c r="O6" s="27" t="str">
+      <x:c r="P6" t="str">
         <x:v>西班牙语示例</x:v>
       </x:c>
     </x:row>
@@ -880,17 +888,18 @@
       <x:c r="J7" s="27" t="str">
         <x:v>报错;步骤</x:v>
       </x:c>
-      <x:c r="K7" s="27" t="str">
+      <x:c r="K7" s="27"/>
+      <x:c r="L7" s="27" t="str">
         <x:v>DICloak</x:v>
       </x:c>
-      <x:c r="L7" s="27" t="str"/>
-      <x:c r="M7" s="27" t="str">
+      <x:c r="M7" s="27"/>
+      <x:c r="N7" s="27" t="str">
         <x:v>请提供报错文本和复现步骤。</x:v>
       </x:c>
-      <x:c r="N7" s="27" t="str">
+      <x:c r="O7" s="27" t="str">
         <x:v>应追问;产品串线</x:v>
       </x:c>
-      <x:c r="O7" s="27" t="str">
+      <x:c r="P7" t="str">
         <x:v>信息不足时应追问</x:v>
       </x:c>
     </x:row>
@@ -921,17 +930,18 @@
       <x:c r="J8" s="29" t="str">
         <x:v>需进一步确认</x:v>
       </x:c>
-      <x:c r="K8" s="29" t="str">
+      <x:c r="K8" s="29"/>
+      <x:c r="L8" s="29" t="str">
         <x:v>保证;根据知识库;FAQ_ID</x:v>
       </x:c>
-      <x:c r="L8" s="29" t="str"/>
-      <x:c r="M8" s="29" t="str">
+      <x:c r="M8" s="29"/>
+      <x:c r="N8" s="29" t="str">
         <x:v>该问题需进一步确认，不能作出保证。</x:v>
       </x:c>
-      <x:c r="N8" s="29" t="str">
+      <x:c r="O8" s="29" t="str">
         <x:v>无知识;内部表达</x:v>
       </x:c>
-      <x:c r="O8" s="29" t="str">
+      <x:c r="P8" t="str">
         <x:v>无知识不得编造</x:v>
       </x:c>
     </x:row>
@@ -955,7 +965,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf38dc7c9027f4af3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R352fd5df8c0441f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>